<commit_message>
previo a pruebas con classroom fake
</commit_message>
<xml_diff>
--- a/config/Rubric.xlsx
+++ b/config/Rubric.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="0" windowWidth="16940" windowHeight="21600" tabRatio="500"/>
+    <workbookView xWindow="-38400" yWindow="0" windowWidth="16940" windowHeight="21600" tabRatio="500" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="CONFIG" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="657">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="658">
   <si>
     <t>General information</t>
   </si>
@@ -2008,6 +2008,9 @@
   </si>
   <si>
     <t>1.0.0</t>
+  </si>
+  <si>
+    <t>Sistema híbrido de evaluación académica asistida por IA con control final del profesor</t>
   </si>
 </sst>
 </file>
@@ -10174,7 +10177,7 @@
   <sheetPr enableFormatConditionsCalculation="0">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A3:J94"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -10182,6 +10185,11 @@
     <col min="3" max="3" width="33.6640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E1" s="14" t="s">
+        <v>657</v>
+      </c>
+    </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E3" s="3" t="s">
         <v>400</v>

</xml_diff>